<commit_message>
feat(data): add 32 verified downstream steel indicators to A03 data map
</commit_message>
<xml_diff>
--- a/outputs/阶段A_框架初版/A03_数据地图.xlsx
+++ b/outputs/阶段A_框架初版/A03_数据地图.xlsx
@@ -185,7 +185,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Register1" displayName="Register1" ref="A5:R78" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Register1" displayName="Register1" ref="A5:R110" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <tableColumns count="18">
     <tableColumn id="1" name="变量ID"/>
     <tableColumn id="2" name="模块"/>
@@ -6669,132 +6669,2692 @@
       </c>
     </row>
     <row r="79">
-      <c r="L79" s="15" t="n"/>
-      <c r="M79" s="15" t="n"/>
+      <c r="A79" s="9" t="inlineStr">
+        <is>
+          <t>B01</t>
+        </is>
+      </c>
+      <c r="B79" s="9" t="inlineStr">
+        <is>
+          <t>现货</t>
+        </is>
+      </c>
+      <c r="C79" s="9" t="inlineStr">
+        <is>
+          <t>唐山方坯现货价格</t>
+        </is>
+      </c>
+      <c r="D79" s="9" t="inlineStr">
+        <is>
+          <t>初级成材价格基准</t>
+        </is>
+      </c>
+      <c r="E79" s="9" t="inlineStr">
+        <is>
+          <t>日</t>
+        </is>
+      </c>
+      <c r="F79" s="9" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G79" s="9" t="inlineStr">
+        <is>
+          <t>元/吨</t>
+        </is>
+      </c>
+      <c r="H79" s="9" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I79" s="9" t="inlineStr">
+        <is>
+          <t>必须</t>
+        </is>
+      </c>
+      <c r="J79" s="9" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K79" s="9" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
+      <c r="L79" s="14" t="n"/>
+      <c r="M79" s="14" t="n"/>
+      <c r="N79" s="9" t="inlineStr">
+        <is>
+          <t>S0143493</t>
+        </is>
+      </c>
+      <c r="O79" s="9" t="inlineStr">
+        <is>
+          <t>中国:唐山:价格:方坯(Q235)</t>
+        </is>
+      </c>
+      <c r="P79" s="9" t="inlineStr">
+        <is>
+          <t>2007-06-25</t>
+        </is>
+      </c>
+      <c r="Q79" s="9" t="inlineStr">
+        <is>
+          <t>每个交易日更新；日频有效</t>
+        </is>
+      </c>
+      <c r="R79" s="9" t="inlineStr">
+        <is>
+          <t>初级材现货基准价格，调坯轧材最核心成本线</t>
+        </is>
+      </c>
     </row>
     <row r="80">
-      <c r="L80" s="15" t="n"/>
-      <c r="M80" s="15" t="n"/>
+      <c r="A80" s="9" t="inlineStr">
+        <is>
+          <t>B02</t>
+        </is>
+      </c>
+      <c r="B80" s="9" t="inlineStr">
+        <is>
+          <t>总供应</t>
+        </is>
+      </c>
+      <c r="C80" s="9" t="inlineStr">
+        <is>
+          <t>唐山钢坯库存量</t>
+        </is>
+      </c>
+      <c r="D80" s="9" t="inlineStr">
+        <is>
+          <t>初级材蓄水池(总库存)</t>
+        </is>
+      </c>
+      <c r="E80" s="9" t="inlineStr">
+        <is>
+          <t>周</t>
+        </is>
+      </c>
+      <c r="F80" s="9" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G80" s="9" t="inlineStr">
+        <is>
+          <t>万吨</t>
+        </is>
+      </c>
+      <c r="H80" s="9" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I80" s="9" t="inlineStr">
+        <is>
+          <t>必须</t>
+        </is>
+      </c>
+      <c r="J80" s="9" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K80" s="9" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
+      <c r="L80" s="14" t="n"/>
+      <c r="M80" s="14" t="n"/>
+      <c r="N80" s="9" t="inlineStr">
+        <is>
+          <t>S5707600</t>
+        </is>
+      </c>
+      <c r="O80" s="9" t="inlineStr">
+        <is>
+          <t>中国:唐山:库存量:钢坯</t>
+        </is>
+      </c>
+      <c r="P80" s="9" t="inlineStr">
+        <is>
+          <t>2011-06-24</t>
+        </is>
+      </c>
+      <c r="Q80" s="9" t="inlineStr">
+        <is>
+          <t>周四发布；周频有效</t>
+        </is>
+      </c>
+      <c r="R80" s="9" t="inlineStr">
+        <is>
+          <t>钢之家统计唐山全口径钢坯仓储总库存</t>
+        </is>
+      </c>
     </row>
     <row r="81">
-      <c r="L81" s="15" t="n"/>
-      <c r="M81" s="15" t="n"/>
+      <c r="A81" s="9" t="inlineStr">
+        <is>
+          <t>B03</t>
+        </is>
+      </c>
+      <c r="B81" s="9" t="inlineStr">
+        <is>
+          <t>总供应</t>
+        </is>
+      </c>
+      <c r="C81" s="9" t="inlineStr">
+        <is>
+          <t>唐山钢坯象屿正丰库库存</t>
+        </is>
+      </c>
+      <c r="D81" s="9" t="inlineStr">
+        <is>
+          <t>核心仓储库存</t>
+        </is>
+      </c>
+      <c r="E81" s="9" t="inlineStr">
+        <is>
+          <t>周</t>
+        </is>
+      </c>
+      <c r="F81" s="9" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G81" s="9" t="inlineStr">
+        <is>
+          <t>万吨</t>
+        </is>
+      </c>
+      <c r="H81" s="9" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I81" s="9" t="inlineStr">
+        <is>
+          <t>候选</t>
+        </is>
+      </c>
+      <c r="J81" s="9" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K81" s="9" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
+      <c r="L81" s="14" t="n"/>
+      <c r="M81" s="14" t="n"/>
+      <c r="N81" s="9" t="inlineStr">
+        <is>
+          <t>S5707595</t>
+        </is>
+      </c>
+      <c r="O81" s="9" t="inlineStr">
+        <is>
+          <t>中国:唐山:库存量:钢坯:象屿正丰库</t>
+        </is>
+      </c>
+      <c r="P81" s="9" t="inlineStr">
+        <is>
+          <t>2017-06-02</t>
+        </is>
+      </c>
+      <c r="Q81" s="9" t="inlineStr">
+        <is>
+          <t>周四发布；周频有效</t>
+        </is>
+      </c>
+      <c r="R81" s="9" t="inlineStr">
+        <is>
+          <t>唐山核心交割与现货集散仓库</t>
+        </is>
+      </c>
     </row>
     <row r="82">
-      <c r="L82" s="15" t="n"/>
-      <c r="M82" s="15" t="n"/>
+      <c r="A82" s="9" t="inlineStr">
+        <is>
+          <t>B04</t>
+        </is>
+      </c>
+      <c r="B82" s="9" t="inlineStr">
+        <is>
+          <t>总供应</t>
+        </is>
+      </c>
+      <c r="C82" s="9" t="inlineStr">
+        <is>
+          <t>唐山钢坯京唐港库存</t>
+        </is>
+      </c>
+      <c r="D82" s="9" t="inlineStr">
+        <is>
+          <t>港口中转库存</t>
+        </is>
+      </c>
+      <c r="E82" s="9" t="inlineStr">
+        <is>
+          <t>周</t>
+        </is>
+      </c>
+      <c r="F82" s="9" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G82" s="9" t="inlineStr">
+        <is>
+          <t>万吨</t>
+        </is>
+      </c>
+      <c r="H82" s="9" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I82" s="9" t="inlineStr">
+        <is>
+          <t>候选</t>
+        </is>
+      </c>
+      <c r="J82" s="9" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K82" s="9" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
+      <c r="L82" s="14" t="n"/>
+      <c r="M82" s="14" t="n"/>
+      <c r="N82" s="9" t="inlineStr">
+        <is>
+          <t>S5707596</t>
+        </is>
+      </c>
+      <c r="O82" s="9" t="inlineStr">
+        <is>
+          <t>中国:唐山:库存量:钢坯:京唐港</t>
+        </is>
+      </c>
+      <c r="P82" s="9" t="inlineStr">
+        <is>
+          <t>2017-06-02</t>
+        </is>
+      </c>
+      <c r="Q82" s="9" t="inlineStr">
+        <is>
+          <t>周四发布；周频有效</t>
+        </is>
+      </c>
+      <c r="R82" s="9" t="inlineStr">
+        <is>
+          <t>港口钢坯中转与南下发运库存</t>
+        </is>
+      </c>
     </row>
     <row r="83">
-      <c r="L83" s="15" t="n"/>
-      <c r="M83" s="15" t="n"/>
+      <c r="A83" s="9" t="inlineStr">
+        <is>
+          <t>B05</t>
+        </is>
+      </c>
+      <c r="B83" s="9" t="inlineStr">
+        <is>
+          <t>总供应</t>
+        </is>
+      </c>
+      <c r="C83" s="9" t="inlineStr">
+        <is>
+          <t>重点企业钢坯累计产量</t>
+        </is>
+      </c>
+      <c r="D83" s="9" t="inlineStr">
+        <is>
+          <t>钢厂钢坯外发产出</t>
+        </is>
+      </c>
+      <c r="E83" s="9" t="inlineStr">
+        <is>
+          <t>月</t>
+        </is>
+      </c>
+      <c r="F83" s="9" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G83" s="9" t="inlineStr">
+        <is>
+          <t>万吨</t>
+        </is>
+      </c>
+      <c r="H83" s="9" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I83" s="9" t="inlineStr">
+        <is>
+          <t>候选</t>
+        </is>
+      </c>
+      <c r="J83" s="9" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K83" s="9" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
+      <c r="L83" s="14" t="n"/>
+      <c r="M83" s="14" t="n"/>
+      <c r="N83" s="9" t="inlineStr">
+        <is>
+          <t>S0114053</t>
+        </is>
+      </c>
+      <c r="O83" s="9" t="inlineStr">
+        <is>
+          <t>中国:产量:钢坯:重点企业:累计值</t>
+        </is>
+      </c>
+      <c r="P83" s="9" t="inlineStr">
+        <is>
+          <t>2005-01-31</t>
+        </is>
+      </c>
+      <c r="Q83" s="9" t="inlineStr">
+        <is>
+          <t>月度发布；月频有效</t>
+        </is>
+      </c>
+      <c r="R83" s="9" t="inlineStr">
+        <is>
+          <t>中钢协重点钢铁企业钢坯外售与调拨累计量</t>
+        </is>
+      </c>
     </row>
     <row r="84">
-      <c r="L84" s="15" t="n"/>
-      <c r="M84" s="15" t="n"/>
+      <c r="A84" s="9" t="inlineStr">
+        <is>
+          <t>B06</t>
+        </is>
+      </c>
+      <c r="B84" s="9" t="inlineStr">
+        <is>
+          <t>总供应</t>
+        </is>
+      </c>
+      <c r="C84" s="9" t="inlineStr">
+        <is>
+          <t>唐山调坯带钢开工率</t>
+        </is>
+      </c>
+      <c r="D84" s="9" t="inlineStr">
+        <is>
+          <t>调坯轧材负荷强度</t>
+        </is>
+      </c>
+      <c r="E84" s="9" t="inlineStr">
+        <is>
+          <t>周</t>
+        </is>
+      </c>
+      <c r="F84" s="9" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G84" s="9" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H84" s="9" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I84" s="9" t="inlineStr">
+        <is>
+          <t>候选</t>
+        </is>
+      </c>
+      <c r="J84" s="9" t="inlineStr">
+        <is>
+          <t>代理变量</t>
+        </is>
+      </c>
+      <c r="K84" s="9" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
+      <c r="L84" s="14" t="n"/>
+      <c r="M84" s="14" t="n"/>
+      <c r="N84" s="9" t="inlineStr">
+        <is>
+          <t>Y7026272</t>
+        </is>
+      </c>
+      <c r="O84" s="9" t="inlineStr">
+        <is>
+          <t>富宝:唐山:开工率:带钢(232以上)</t>
+        </is>
+      </c>
+      <c r="P84" s="9" t="inlineStr">
+        <is>
+          <t>2018-03-02</t>
+        </is>
+      </c>
+      <c r="Q84" s="9" t="inlineStr">
+        <is>
+          <t>周四发布；周频有效</t>
+        </is>
+      </c>
+      <c r="R84" s="9" t="inlineStr">
+        <is>
+          <t>反映唐山调坯轧材企业实际开工率，衡量对钢坯的拉动力</t>
+        </is>
+      </c>
     </row>
     <row r="85">
-      <c r="L85" s="15" t="n"/>
-      <c r="M85" s="15" t="n"/>
+      <c r="A85" s="9" t="inlineStr">
+        <is>
+          <t>W01</t>
+        </is>
+      </c>
+      <c r="B85" s="9" t="inlineStr">
+        <is>
+          <t>螺纹</t>
+        </is>
+      </c>
+      <c r="C85" s="9" t="inlineStr">
+        <is>
+          <t>线材周产量</t>
+        </is>
+      </c>
+      <c r="D85" s="9" t="inlineStr">
+        <is>
+          <t>长材/线材品种供应</t>
+        </is>
+      </c>
+      <c r="E85" s="9" t="inlineStr">
+        <is>
+          <t>周</t>
+        </is>
+      </c>
+      <c r="F85" s="9" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G85" s="9" t="inlineStr">
+        <is>
+          <t>万吨</t>
+        </is>
+      </c>
+      <c r="H85" s="9" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I85" s="9" t="inlineStr">
+        <is>
+          <t>必须</t>
+        </is>
+      </c>
+      <c r="J85" s="9" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K85" s="9" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
+      <c r="L85" s="14" t="n"/>
+      <c r="M85" s="14" t="n"/>
+      <c r="N85" s="9" t="inlineStr">
+        <is>
+          <t>S5713331</t>
+        </is>
+      </c>
+      <c r="O85" s="9" t="inlineStr">
+        <is>
+          <t>中国:产量:线材:主要钢厂</t>
+        </is>
+      </c>
+      <c r="P85" s="9" t="inlineStr">
+        <is>
+          <t>2015-02-27</t>
+        </is>
+      </c>
+      <c r="Q85" s="9" t="inlineStr">
+        <is>
+          <t>周五发布；周频有效</t>
+        </is>
+      </c>
+      <c r="R85" s="9" t="inlineStr">
+        <is>
+          <t>主要钢厂线材周产量口径</t>
+        </is>
+      </c>
     </row>
     <row r="86">
-      <c r="L86" s="15" t="n"/>
-      <c r="M86" s="15" t="n"/>
+      <c r="A86" s="9" t="inlineStr">
+        <is>
+          <t>W02</t>
+        </is>
+      </c>
+      <c r="B86" s="9" t="inlineStr">
+        <is>
+          <t>螺纹</t>
+        </is>
+      </c>
+      <c r="C86" s="9" t="inlineStr">
+        <is>
+          <t>线材产能利用率</t>
+        </is>
+      </c>
+      <c r="D86" s="9" t="inlineStr">
+        <is>
+          <t>线材生产线负荷</t>
+        </is>
+      </c>
+      <c r="E86" s="9" t="inlineStr">
+        <is>
+          <t>周</t>
+        </is>
+      </c>
+      <c r="F86" s="9" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G86" s="9" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H86" s="9" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I86" s="9" t="inlineStr">
+        <is>
+          <t>候选</t>
+        </is>
+      </c>
+      <c r="J86" s="9" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K86" s="9" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
+      <c r="L86" s="14" t="n"/>
+      <c r="M86" s="14" t="n"/>
+      <c r="N86" s="9" t="inlineStr">
+        <is>
+          <t>S5713335</t>
+        </is>
+      </c>
+      <c r="O86" s="9" t="inlineStr">
+        <is>
+          <t>中国:产能利用率:线材:主要钢厂</t>
+        </is>
+      </c>
+      <c r="P86" s="9" t="inlineStr">
+        <is>
+          <t>2015-02-27</t>
+        </is>
+      </c>
+      <c r="Q86" s="9" t="inlineStr">
+        <is>
+          <t>周五发布；周频有效</t>
+        </is>
+      </c>
+      <c r="R86" s="9" t="inlineStr">
+        <is>
+          <t>主要钢厂线材轧线产能利用率</t>
+        </is>
+      </c>
     </row>
     <row r="87">
-      <c r="L87" s="15" t="n"/>
-      <c r="M87" s="15" t="n"/>
+      <c r="A87" s="9" t="inlineStr">
+        <is>
+          <t>W03</t>
+        </is>
+      </c>
+      <c r="B87" s="9" t="inlineStr">
+        <is>
+          <t>螺纹</t>
+        </is>
+      </c>
+      <c r="C87" s="9" t="inlineStr">
+        <is>
+          <t>线材社会库存</t>
+        </is>
+      </c>
+      <c r="D87" s="9" t="inlineStr">
+        <is>
+          <t>流通环节线材库存</t>
+        </is>
+      </c>
+      <c r="E87" s="9" t="inlineStr">
+        <is>
+          <t>周</t>
+        </is>
+      </c>
+      <c r="F87" s="9" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G87" s="9" t="inlineStr">
+        <is>
+          <t>万吨</t>
+        </is>
+      </c>
+      <c r="H87" s="9" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I87" s="9" t="inlineStr">
+        <is>
+          <t>必须</t>
+        </is>
+      </c>
+      <c r="J87" s="9" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K87" s="9" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
+      <c r="L87" s="14" t="n"/>
+      <c r="M87" s="14" t="n"/>
+      <c r="N87" s="9" t="inlineStr">
+        <is>
+          <t>N5497850</t>
+        </is>
+      </c>
+      <c r="O87" s="9" t="inlineStr">
+        <is>
+          <t>中国:社会库存量:线材</t>
+        </is>
+      </c>
+      <c r="P87" s="9" t="inlineStr">
+        <is>
+          <t>2020-01-20</t>
+        </is>
+      </c>
+      <c r="Q87" s="9" t="inlineStr">
+        <is>
+          <t>周四发布；周频有效</t>
+        </is>
+      </c>
+      <c r="R87" s="9" t="inlineStr">
+        <is>
+          <t>全国主流城市线材流通社会库存</t>
+        </is>
+      </c>
     </row>
     <row r="88">
-      <c r="L88" s="15" t="n"/>
-      <c r="M88" s="15" t="n"/>
+      <c r="A88" s="9" t="inlineStr">
+        <is>
+          <t>W04</t>
+        </is>
+      </c>
+      <c r="B88" s="9" t="inlineStr">
+        <is>
+          <t>螺纹</t>
+        </is>
+      </c>
+      <c r="C88" s="9" t="inlineStr">
+        <is>
+          <t>线材钢厂库存</t>
+        </is>
+      </c>
+      <c r="D88" s="9" t="inlineStr">
+        <is>
+          <t>钢厂环节线材库存</t>
+        </is>
+      </c>
+      <c r="E88" s="9" t="inlineStr">
+        <is>
+          <t>周</t>
+        </is>
+      </c>
+      <c r="F88" s="9" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G88" s="9" t="inlineStr">
+        <is>
+          <t>万吨</t>
+        </is>
+      </c>
+      <c r="H88" s="9" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I88" s="9" t="inlineStr">
+        <is>
+          <t>必须</t>
+        </is>
+      </c>
+      <c r="J88" s="9" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K88" s="9" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
+      <c r="L88" s="14" t="n"/>
+      <c r="M88" s="14" t="n"/>
+      <c r="N88" s="9" t="inlineStr">
+        <is>
+          <t>N2859772</t>
+        </is>
+      </c>
+      <c r="O88" s="9" t="inlineStr">
+        <is>
+          <t>中国:库存量:线材:主要钢厂</t>
+        </is>
+      </c>
+      <c r="P88" s="9" t="inlineStr">
+        <is>
+          <t>2020-02-07</t>
+        </is>
+      </c>
+      <c r="Q88" s="9" t="inlineStr">
+        <is>
+          <t>周五发布；周频有效</t>
+        </is>
+      </c>
+      <c r="R88" s="9" t="inlineStr">
+        <is>
+          <t>主要钢厂线材周度厂库 (备选S5713338)</t>
+        </is>
+      </c>
     </row>
     <row r="89">
-      <c r="L89" s="15" t="n"/>
-      <c r="M89" s="15" t="n"/>
+      <c r="A89" s="9" t="inlineStr">
+        <is>
+          <t>W05</t>
+        </is>
+      </c>
+      <c r="B89" s="9" t="inlineStr">
+        <is>
+          <t>螺纹</t>
+        </is>
+      </c>
+      <c r="C89" s="9" t="inlineStr">
+        <is>
+          <t>线材表观需求量</t>
+        </is>
+      </c>
+      <c r="D89" s="9" t="inlineStr">
+        <is>
+          <t>线材终端消费代理</t>
+        </is>
+      </c>
+      <c r="E89" s="9" t="inlineStr">
+        <is>
+          <t>周</t>
+        </is>
+      </c>
+      <c r="F89" s="9" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G89" s="9" t="inlineStr">
+        <is>
+          <t>万吨</t>
+        </is>
+      </c>
+      <c r="H89" s="9" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I89" s="9" t="inlineStr">
+        <is>
+          <t>必须</t>
+        </is>
+      </c>
+      <c r="J89" s="9" t="inlineStr">
+        <is>
+          <t>计算代理</t>
+        </is>
+      </c>
+      <c r="K89" s="9" t="inlineStr">
+        <is>
+          <t>计算</t>
+        </is>
+      </c>
+      <c r="L89" s="14" t="n"/>
+      <c r="M89" s="14" t="n"/>
+      <c r="N89" s="9" t="inlineStr">
+        <is>
+          <t>Y1232969</t>
+        </is>
+      </c>
+      <c r="O89" s="9" t="inlineStr">
+        <is>
+          <t>中国:表观需求量:线材</t>
+        </is>
+      </c>
+      <c r="P89" s="9" t="inlineStr">
+        <is>
+          <t>2015-08-07</t>
+        </is>
+      </c>
+      <c r="Q89" s="9" t="inlineStr">
+        <is>
+          <t>周五发布；周频有效</t>
+        </is>
+      </c>
+      <c r="R89" s="9" t="inlineStr">
+        <is>
+          <t>周度官方反推表需序列</t>
+        </is>
+      </c>
     </row>
     <row r="90">
-      <c r="L90" s="15" t="n"/>
-      <c r="M90" s="15" t="n"/>
+      <c r="A90" s="9" t="inlineStr">
+        <is>
+          <t>W06</t>
+        </is>
+      </c>
+      <c r="B90" s="9" t="inlineStr">
+        <is>
+          <t>现货</t>
+        </is>
+      </c>
+      <c r="C90" s="9" t="inlineStr">
+        <is>
+          <t>上海高线现货价格</t>
+        </is>
+      </c>
+      <c r="D90" s="9" t="inlineStr">
+        <is>
+          <t>长材高线现实价格</t>
+        </is>
+      </c>
+      <c r="E90" s="9" t="inlineStr">
+        <is>
+          <t>日</t>
+        </is>
+      </c>
+      <c r="F90" s="9" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G90" s="9" t="inlineStr">
+        <is>
+          <t>元/吨</t>
+        </is>
+      </c>
+      <c r="H90" s="9" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I90" s="9" t="inlineStr">
+        <is>
+          <t>候选</t>
+        </is>
+      </c>
+      <c r="J90" s="9" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K90" s="9" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
+      <c r="L90" s="14" t="n"/>
+      <c r="M90" s="14" t="n"/>
+      <c r="N90" s="9" t="inlineStr">
+        <is>
+          <t>S5707104</t>
+        </is>
+      </c>
+      <c r="O90" s="9" t="inlineStr">
+        <is>
+          <t>中国:上海:价格:高线(8,HPB300)</t>
+        </is>
+      </c>
+      <c r="P90" s="9" t="inlineStr">
+        <is>
+          <t>2007-01-08</t>
+        </is>
+      </c>
+      <c r="Q90" s="9" t="inlineStr">
+        <is>
+          <t>每个交易日下午更新；日频有效</t>
+        </is>
+      </c>
+      <c r="R90" s="9" t="inlineStr">
+        <is>
+          <t>上海HPB300 8mm高线现货基准日价</t>
+        </is>
+      </c>
     </row>
     <row r="91">
-      <c r="L91" s="15" t="n"/>
-      <c r="M91" s="15" t="n"/>
+      <c r="A91" s="9" t="inlineStr">
+        <is>
+          <t>CR01</t>
+        </is>
+      </c>
+      <c r="B91" s="9" t="inlineStr">
+        <is>
+          <t>热卷</t>
+        </is>
+      </c>
+      <c r="C91" s="9" t="inlineStr">
+        <is>
+          <t>冷轧板卷周产量</t>
+        </is>
+      </c>
+      <c r="D91" s="9" t="inlineStr">
+        <is>
+          <t>热卷深度加工产出</t>
+        </is>
+      </c>
+      <c r="E91" s="9" t="inlineStr">
+        <is>
+          <t>周</t>
+        </is>
+      </c>
+      <c r="F91" s="9" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G91" s="9" t="inlineStr">
+        <is>
+          <t>万吨</t>
+        </is>
+      </c>
+      <c r="H91" s="9" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I91" s="9" t="inlineStr">
+        <is>
+          <t>必须</t>
+        </is>
+      </c>
+      <c r="J91" s="9" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K91" s="9" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
+      <c r="L91" s="14" t="n"/>
+      <c r="M91" s="14" t="n"/>
+      <c r="N91" s="9" t="inlineStr">
+        <is>
+          <t>U9895886</t>
+        </is>
+      </c>
+      <c r="O91" s="9" t="inlineStr">
+        <is>
+          <t>中国:产量:冷轧板卷:主要钢厂</t>
+        </is>
+      </c>
+      <c r="P91" s="9" t="inlineStr">
+        <is>
+          <t>2020-02-07</t>
+        </is>
+      </c>
+      <c r="Q91" s="9" t="inlineStr">
+        <is>
+          <t>周五发布；周频有效</t>
+        </is>
+      </c>
+      <c r="R91" s="9" t="inlineStr">
+        <is>
+          <t>热卷向冷轧转化的主要钢厂周产量，直接反映热卷的下游消化</t>
+        </is>
+      </c>
     </row>
     <row r="92">
-      <c r="L92" s="15" t="n"/>
-      <c r="M92" s="15" t="n"/>
+      <c r="A92" s="9" t="inlineStr">
+        <is>
+          <t>CR02</t>
+        </is>
+      </c>
+      <c r="B92" s="9" t="inlineStr">
+        <is>
+          <t>热卷</t>
+        </is>
+      </c>
+      <c r="C92" s="9" t="inlineStr">
+        <is>
+          <t>冷轧板卷社会库存</t>
+        </is>
+      </c>
+      <c r="D92" s="9" t="inlineStr">
+        <is>
+          <t>流通环节冷轧库存</t>
+        </is>
+      </c>
+      <c r="E92" s="9" t="inlineStr">
+        <is>
+          <t>周</t>
+        </is>
+      </c>
+      <c r="F92" s="9" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G92" s="9" t="inlineStr">
+        <is>
+          <t>万吨</t>
+        </is>
+      </c>
+      <c r="H92" s="9" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I92" s="9" t="inlineStr">
+        <is>
+          <t>必须</t>
+        </is>
+      </c>
+      <c r="J92" s="9" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K92" s="9" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
+      <c r="L92" s="14" t="n"/>
+      <c r="M92" s="14" t="n"/>
+      <c r="N92" s="9" t="inlineStr">
+        <is>
+          <t>W2000685</t>
+        </is>
+      </c>
+      <c r="O92" s="9" t="inlineStr">
+        <is>
+          <t>中国:社会库存量:冷轧板卷</t>
+        </is>
+      </c>
+      <c r="P92" s="9" t="inlineStr">
+        <is>
+          <t>2020-01-20</t>
+        </is>
+      </c>
+      <c r="Q92" s="9" t="inlineStr">
+        <is>
+          <t>周四发布；周频有效</t>
+        </is>
+      </c>
+      <c r="R92" s="9" t="inlineStr">
+        <is>
+          <t>主流城市冷轧板卷社会流通库存</t>
+        </is>
+      </c>
     </row>
     <row r="93">
-      <c r="L93" s="15" t="n"/>
-      <c r="M93" s="15" t="n"/>
+      <c r="A93" s="9" t="inlineStr">
+        <is>
+          <t>CR03</t>
+        </is>
+      </c>
+      <c r="B93" s="9" t="inlineStr">
+        <is>
+          <t>热卷</t>
+        </is>
+      </c>
+      <c r="C93" s="9" t="inlineStr">
+        <is>
+          <t>冷轧板卷钢厂库存</t>
+        </is>
+      </c>
+      <c r="D93" s="9" t="inlineStr">
+        <is>
+          <t>钢厂环节冷轧库存</t>
+        </is>
+      </c>
+      <c r="E93" s="9" t="inlineStr">
+        <is>
+          <t>周</t>
+        </is>
+      </c>
+      <c r="F93" s="9" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G93" s="9" t="inlineStr">
+        <is>
+          <t>万吨</t>
+        </is>
+      </c>
+      <c r="H93" s="9" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I93" s="9" t="inlineStr">
+        <is>
+          <t>必须</t>
+        </is>
+      </c>
+      <c r="J93" s="9" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K93" s="9" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
+      <c r="L93" s="14" t="n"/>
+      <c r="M93" s="14" t="n"/>
+      <c r="N93" s="9" t="inlineStr">
+        <is>
+          <t>V9343799</t>
+        </is>
+      </c>
+      <c r="O93" s="9" t="inlineStr">
+        <is>
+          <t>中国:库存量:冷轧板卷:主要钢厂</t>
+        </is>
+      </c>
+      <c r="P93" s="9" t="inlineStr">
+        <is>
+          <t>2020-02-07</t>
+        </is>
+      </c>
+      <c r="Q93" s="9" t="inlineStr">
+        <is>
+          <t>周五发布；周频有效</t>
+        </is>
+      </c>
+      <c r="R93" s="9" t="inlineStr">
+        <is>
+          <t>主要钢厂冷轧板卷周度厂库</t>
+        </is>
+      </c>
     </row>
     <row r="94">
-      <c r="L94" s="15" t="n"/>
-      <c r="M94" s="15" t="n"/>
+      <c r="A94" s="9" t="inlineStr">
+        <is>
+          <t>CR04</t>
+        </is>
+      </c>
+      <c r="B94" s="9" t="inlineStr">
+        <is>
+          <t>热卷</t>
+        </is>
+      </c>
+      <c r="C94" s="9" t="inlineStr">
+        <is>
+          <t>冷轧板卷月度表观消费</t>
+        </is>
+      </c>
+      <c r="D94" s="9" t="inlineStr">
+        <is>
+          <t>板材终端消费代理</t>
+        </is>
+      </c>
+      <c r="E94" s="9" t="inlineStr">
+        <is>
+          <t>月</t>
+        </is>
+      </c>
+      <c r="F94" s="9" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G94" s="9" t="inlineStr">
+        <is>
+          <t>万吨</t>
+        </is>
+      </c>
+      <c r="H94" s="9" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I94" s="9" t="inlineStr">
+        <is>
+          <t>候选</t>
+        </is>
+      </c>
+      <c r="J94" s="9" t="inlineStr">
+        <is>
+          <t>计算代理</t>
+        </is>
+      </c>
+      <c r="K94" s="9" t="inlineStr">
+        <is>
+          <t>计算</t>
+        </is>
+      </c>
+      <c r="L94" s="14" t="n"/>
+      <c r="M94" s="14" t="n"/>
+      <c r="N94" s="9" t="inlineStr">
+        <is>
+          <t>S5707786</t>
+        </is>
+      </c>
+      <c r="O94" s="9" t="inlineStr">
+        <is>
+          <t>中国:表观消费量:冷轧薄板</t>
+        </is>
+      </c>
+      <c r="P94" s="9" t="inlineStr">
+        <is>
+          <t>2008-01-31</t>
+        </is>
+      </c>
+      <c r="Q94" s="9" t="inlineStr">
+        <is>
+          <t>月度发布；月频有效</t>
+        </is>
+      </c>
+      <c r="R94" s="9" t="inlineStr">
+        <is>
+          <t>官方月度冷轧表观消费反推</t>
+        </is>
+      </c>
     </row>
     <row r="95">
-      <c r="L95" s="15" t="n"/>
-      <c r="M95" s="15" t="n"/>
+      <c r="A95" s="9" t="inlineStr">
+        <is>
+          <t>CR05</t>
+        </is>
+      </c>
+      <c r="B95" s="9" t="inlineStr">
+        <is>
+          <t>现货</t>
+        </is>
+      </c>
+      <c r="C95" s="9" t="inlineStr">
+        <is>
+          <t>上海冷轧板卷现货价格</t>
+        </is>
+      </c>
+      <c r="D95" s="9" t="inlineStr">
+        <is>
+          <t>冷轧现实价格基准</t>
+        </is>
+      </c>
+      <c r="E95" s="9" t="inlineStr">
+        <is>
+          <t>日</t>
+        </is>
+      </c>
+      <c r="F95" s="9" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G95" s="9" t="inlineStr">
+        <is>
+          <t>元/吨</t>
+        </is>
+      </c>
+      <c r="H95" s="9" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I95" s="9" t="inlineStr">
+        <is>
+          <t>必须</t>
+        </is>
+      </c>
+      <c r="J95" s="9" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K95" s="9" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
+      <c r="L95" s="14" t="n"/>
+      <c r="M95" s="14" t="n"/>
+      <c r="N95" s="9" t="inlineStr">
+        <is>
+          <t>S0033155</t>
+        </is>
+      </c>
+      <c r="O95" s="9" t="inlineStr">
+        <is>
+          <t>中国:上海:价格:冷轧板卷(1.0mm)</t>
+        </is>
+      </c>
+      <c r="P95" s="9" t="inlineStr">
+        <is>
+          <t>2002-01-21</t>
+        </is>
+      </c>
+      <c r="Q95" s="9" t="inlineStr">
+        <is>
+          <t>每个交易日下午更新；日频有效</t>
+        </is>
+      </c>
+      <c r="R95" s="9" t="inlineStr">
+        <is>
+          <t>上海1.0mm冷轧现货基准；用于计算冷热价差</t>
+        </is>
+      </c>
     </row>
     <row r="96">
-      <c r="L96" s="15" t="n"/>
-      <c r="M96" s="15" t="n"/>
+      <c r="A96" s="9" t="inlineStr">
+        <is>
+          <t>CR06</t>
+        </is>
+      </c>
+      <c r="B96" s="9" t="inlineStr">
+        <is>
+          <t>现货</t>
+        </is>
+      </c>
+      <c r="C96" s="9" t="inlineStr">
+        <is>
+          <t>冷热现货价差</t>
+        </is>
+      </c>
+      <c r="D96" s="9" t="inlineStr">
+        <is>
+          <t>冷轧深加工附加值与拉动力</t>
+        </is>
+      </c>
+      <c r="E96" s="9" t="inlineStr">
+        <is>
+          <t>日</t>
+        </is>
+      </c>
+      <c r="F96" s="9" t="inlineStr">
+        <is>
+          <t>自有计算</t>
+        </is>
+      </c>
+      <c r="G96" s="9" t="inlineStr">
+        <is>
+          <t>元/吨</t>
+        </is>
+      </c>
+      <c r="H96" s="9" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I96" s="9" t="inlineStr">
+        <is>
+          <t>必须</t>
+        </is>
+      </c>
+      <c r="J96" s="9" t="inlineStr">
+        <is>
+          <t>派生价差</t>
+        </is>
+      </c>
+      <c r="K96" s="9" t="inlineStr">
+        <is>
+          <t>计算</t>
+        </is>
+      </c>
+      <c r="L96" s="14" t="n"/>
+      <c r="M96" s="14" t="n"/>
+      <c r="N96" s="9" t="inlineStr">
+        <is>
+          <t>S0033155 - S0033272</t>
+        </is>
+      </c>
+      <c r="O96" s="9" t="inlineStr">
+        <is>
+          <t>上海冷轧1.0mm减上海热卷4.75mm</t>
+        </is>
+      </c>
+      <c r="P96" s="9" t="inlineStr">
+        <is>
+          <t>2004-10-29</t>
+        </is>
+      </c>
+      <c r="Q96" s="9" t="inlineStr">
+        <is>
+          <t>每个交易日计算；日频有效</t>
+        </is>
+      </c>
+      <c r="R96" s="9" t="inlineStr">
+        <is>
+          <t>衡量冷卷深加工利润空间与冷轧厂对热卷的拉动强度</t>
+        </is>
+      </c>
     </row>
     <row r="97">
-      <c r="L97" s="15" t="n"/>
-      <c r="M97" s="15" t="n"/>
+      <c r="A97" s="9" t="inlineStr">
+        <is>
+          <t>MP01</t>
+        </is>
+      </c>
+      <c r="B97" s="9" t="inlineStr">
+        <is>
+          <t>热卷</t>
+        </is>
+      </c>
+      <c r="C97" s="9" t="inlineStr">
+        <is>
+          <t>中厚板周产量</t>
+        </is>
+      </c>
+      <c r="D97" s="9" t="inlineStr">
+        <is>
+          <t>造船/重型机械板材供应</t>
+        </is>
+      </c>
+      <c r="E97" s="9" t="inlineStr">
+        <is>
+          <t>周</t>
+        </is>
+      </c>
+      <c r="F97" s="9" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G97" s="9" t="inlineStr">
+        <is>
+          <t>万吨</t>
+        </is>
+      </c>
+      <c r="H97" s="9" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I97" s="9" t="inlineStr">
+        <is>
+          <t>必须</t>
+        </is>
+      </c>
+      <c r="J97" s="9" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K97" s="9" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
+      <c r="L97" s="14" t="n"/>
+      <c r="M97" s="14" t="n"/>
+      <c r="N97" s="9" t="inlineStr">
+        <is>
+          <t>D2626009</t>
+        </is>
+      </c>
+      <c r="O97" s="9" t="inlineStr">
+        <is>
+          <t>中国:产量:中厚板:主要钢厂</t>
+        </is>
+      </c>
+      <c r="P97" s="9" t="inlineStr">
+        <is>
+          <t>2020-02-07</t>
+        </is>
+      </c>
+      <c r="Q97" s="9" t="inlineStr">
+        <is>
+          <t>周五发布；周频有效</t>
+        </is>
+      </c>
+      <c r="R97" s="9" t="inlineStr">
+        <is>
+          <t>主要钢厂中厚板周产量</t>
+        </is>
+      </c>
     </row>
     <row r="98">
-      <c r="L98" s="15" t="n"/>
-      <c r="M98" s="15" t="n"/>
+      <c r="A98" s="9" t="inlineStr">
+        <is>
+          <t>MP02</t>
+        </is>
+      </c>
+      <c r="B98" s="9" t="inlineStr">
+        <is>
+          <t>热卷</t>
+        </is>
+      </c>
+      <c r="C98" s="9" t="inlineStr">
+        <is>
+          <t>中厚板社会库存</t>
+        </is>
+      </c>
+      <c r="D98" s="9" t="inlineStr">
+        <is>
+          <t>流通环节中厚板库存</t>
+        </is>
+      </c>
+      <c r="E98" s="9" t="inlineStr">
+        <is>
+          <t>周</t>
+        </is>
+      </c>
+      <c r="F98" s="9" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G98" s="9" t="inlineStr">
+        <is>
+          <t>万吨</t>
+        </is>
+      </c>
+      <c r="H98" s="9" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I98" s="9" t="inlineStr">
+        <is>
+          <t>必须</t>
+        </is>
+      </c>
+      <c r="J98" s="9" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K98" s="9" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
+      <c r="L98" s="14" t="n"/>
+      <c r="M98" s="14" t="n"/>
+      <c r="N98" s="9" t="inlineStr">
+        <is>
+          <t>W6382677</t>
+        </is>
+      </c>
+      <c r="O98" s="9" t="inlineStr">
+        <is>
+          <t>中国:社会库存量:中厚板</t>
+        </is>
+      </c>
+      <c r="P98" s="9" t="inlineStr">
+        <is>
+          <t>2020-01-20</t>
+        </is>
+      </c>
+      <c r="Q98" s="9" t="inlineStr">
+        <is>
+          <t>周四发布；周频有效</t>
+        </is>
+      </c>
+      <c r="R98" s="9" t="inlineStr">
+        <is>
+          <t>主流城市中厚板社会流通库存</t>
+        </is>
+      </c>
     </row>
     <row r="99">
-      <c r="L99" s="15" t="n"/>
-      <c r="M99" s="15" t="n"/>
+      <c r="A99" s="9" t="inlineStr">
+        <is>
+          <t>MP03</t>
+        </is>
+      </c>
+      <c r="B99" s="9" t="inlineStr">
+        <is>
+          <t>热卷</t>
+        </is>
+      </c>
+      <c r="C99" s="9" t="inlineStr">
+        <is>
+          <t>中厚板钢厂库存</t>
+        </is>
+      </c>
+      <c r="D99" s="9" t="inlineStr">
+        <is>
+          <t>钢厂环节中厚板库存</t>
+        </is>
+      </c>
+      <c r="E99" s="9" t="inlineStr">
+        <is>
+          <t>周</t>
+        </is>
+      </c>
+      <c r="F99" s="9" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G99" s="9" t="inlineStr">
+        <is>
+          <t>万吨</t>
+        </is>
+      </c>
+      <c r="H99" s="9" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I99" s="9" t="inlineStr">
+        <is>
+          <t>必须</t>
+        </is>
+      </c>
+      <c r="J99" s="9" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K99" s="9" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
+      <c r="L99" s="14" t="n"/>
+      <c r="M99" s="14" t="n"/>
+      <c r="N99" s="9" t="inlineStr">
+        <is>
+          <t>C1585720</t>
+        </is>
+      </c>
+      <c r="O99" s="9" t="inlineStr">
+        <is>
+          <t>中国:库存量:中厚板:主要钢厂</t>
+        </is>
+      </c>
+      <c r="P99" s="9" t="inlineStr">
+        <is>
+          <t>2020-02-07</t>
+        </is>
+      </c>
+      <c r="Q99" s="9" t="inlineStr">
+        <is>
+          <t>周五发布；周频有效</t>
+        </is>
+      </c>
+      <c r="R99" s="9" t="inlineStr">
+        <is>
+          <t>主要钢厂中厚板周度厂库</t>
+        </is>
+      </c>
     </row>
     <row r="100">
-      <c r="L100" s="15" t="n"/>
-      <c r="M100" s="15" t="n"/>
+      <c r="A100" s="9" t="inlineStr">
+        <is>
+          <t>MP04</t>
+        </is>
+      </c>
+      <c r="B100" s="9" t="inlineStr">
+        <is>
+          <t>现货</t>
+        </is>
+      </c>
+      <c r="C100" s="9" t="inlineStr">
+        <is>
+          <t>全国中厚板均价</t>
+        </is>
+      </c>
+      <c r="D100" s="9" t="inlineStr">
+        <is>
+          <t>中厚板现实价格基准</t>
+        </is>
+      </c>
+      <c r="E100" s="9" t="inlineStr">
+        <is>
+          <t>日</t>
+        </is>
+      </c>
+      <c r="F100" s="9" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G100" s="9" t="inlineStr">
+        <is>
+          <t>元/吨</t>
+        </is>
+      </c>
+      <c r="H100" s="9" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I100" s="9" t="inlineStr">
+        <is>
+          <t>必须</t>
+        </is>
+      </c>
+      <c r="J100" s="9" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K100" s="9" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
+      <c r="L100" s="14" t="n"/>
+      <c r="M100" s="14" t="n"/>
+      <c r="N100" s="9" t="inlineStr">
+        <is>
+          <t>S5709358</t>
+        </is>
+      </c>
+      <c r="O100" s="9" t="inlineStr">
+        <is>
+          <t>中国:价格:中厚板</t>
+        </is>
+      </c>
+      <c r="P100" s="9" t="inlineStr">
+        <is>
+          <t>2014-07-01</t>
+        </is>
+      </c>
+      <c r="Q100" s="9" t="inlineStr">
+        <is>
+          <t>每个交易日更新；日频有效</t>
+        </is>
+      </c>
+      <c r="R100" s="9" t="inlineStr">
+        <is>
+          <t>兰格钢铁网全国中厚板现货均价</t>
+        </is>
+      </c>
     </row>
     <row r="101">
-      <c r="L101" s="15" t="n"/>
-      <c r="M101" s="15" t="n"/>
+      <c r="A101" s="9" t="inlineStr">
+        <is>
+          <t>MP05</t>
+        </is>
+      </c>
+      <c r="B101" s="9" t="inlineStr">
+        <is>
+          <t>现货</t>
+        </is>
+      </c>
+      <c r="C101" s="9" t="inlineStr">
+        <is>
+          <t>上海中厚板现货价格</t>
+        </is>
+      </c>
+      <c r="D101" s="9" t="inlineStr">
+        <is>
+          <t>区域中厚板现货价格</t>
+        </is>
+      </c>
+      <c r="E101" s="9" t="inlineStr">
+        <is>
+          <t>周</t>
+        </is>
+      </c>
+      <c r="F101" s="9" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G101" s="9" t="inlineStr">
+        <is>
+          <t>元/吨</t>
+        </is>
+      </c>
+      <c r="H101" s="9" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I101" s="9" t="inlineStr">
+        <is>
+          <t>候选</t>
+        </is>
+      </c>
+      <c r="J101" s="9" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K101" s="9" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
+      <c r="L101" s="14" t="n"/>
+      <c r="M101" s="14" t="n"/>
+      <c r="N101" s="9" t="inlineStr">
+        <is>
+          <t>W5281756</t>
+        </is>
+      </c>
+      <c r="O101" s="9" t="inlineStr">
+        <is>
+          <t>中国:上海:市场价:中厚板(Q235,20mm)</t>
+        </is>
+      </c>
+      <c r="P101" s="9" t="inlineStr">
+        <is>
+          <t>2020-02-14</t>
+        </is>
+      </c>
+      <c r="Q101" s="9" t="inlineStr">
+        <is>
+          <t>周五发布；周频有效</t>
+        </is>
+      </c>
+      <c r="R101" s="9" t="inlineStr">
+        <is>
+          <t>上海本地20mm中厚板规格周价</t>
+        </is>
+      </c>
     </row>
     <row r="102">
-      <c r="L102" s="15" t="n"/>
-      <c r="M102" s="15" t="n"/>
+      <c r="A102" s="9" t="inlineStr">
+        <is>
+          <t>R06</t>
+        </is>
+      </c>
+      <c r="B102" s="9" t="inlineStr">
+        <is>
+          <t>螺纹</t>
+        </is>
+      </c>
+      <c r="C102" s="9" t="inlineStr">
+        <is>
+          <t>螺纹钢产能利用率</t>
+        </is>
+      </c>
+      <c r="D102" s="9" t="inlineStr">
+        <is>
+          <t>螺纹钢轧线负荷强度</t>
+        </is>
+      </c>
+      <c r="E102" s="9" t="inlineStr">
+        <is>
+          <t>周</t>
+        </is>
+      </c>
+      <c r="F102" s="9" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G102" s="9" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H102" s="9" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I102" s="9" t="inlineStr">
+        <is>
+          <t>必须</t>
+        </is>
+      </c>
+      <c r="J102" s="9" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K102" s="9" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
+      <c r="L102" s="14" t="n"/>
+      <c r="M102" s="14" t="n"/>
+      <c r="N102" s="9" t="inlineStr">
+        <is>
+          <t>S5713311</t>
+        </is>
+      </c>
+      <c r="O102" s="9" t="inlineStr">
+        <is>
+          <t>中国:产能利用率:螺纹钢:主要钢厂</t>
+        </is>
+      </c>
+      <c r="P102" s="9" t="inlineStr">
+        <is>
+          <t>2015-02-27</t>
+        </is>
+      </c>
+      <c r="Q102" s="9" t="inlineStr">
+        <is>
+          <t>周五发布；周频有效</t>
+        </is>
+      </c>
+      <c r="R102" s="9" t="inlineStr">
+        <is>
+          <t>主要钢厂螺纹钢轧线产能利用率，当前在38%低位</t>
+        </is>
+      </c>
     </row>
     <row r="103">
-      <c r="L103" s="15" t="n"/>
-      <c r="M103" s="15" t="n"/>
+      <c r="A103" s="9" t="inlineStr">
+        <is>
+          <t>TOTAL01</t>
+        </is>
+      </c>
+      <c r="B103" s="9" t="inlineStr">
+        <is>
+          <t>总供应</t>
+        </is>
+      </c>
+      <c r="C103" s="9" t="inlineStr">
+        <is>
+          <t>五大钢材主要钢厂周产量合计</t>
+        </is>
+      </c>
+      <c r="D103" s="9" t="inlineStr">
+        <is>
+          <t>主要成材总供给</t>
+        </is>
+      </c>
+      <c r="E103" s="9" t="inlineStr">
+        <is>
+          <t>周</t>
+        </is>
+      </c>
+      <c r="F103" s="9" t="inlineStr">
+        <is>
+          <t>自有计算</t>
+        </is>
+      </c>
+      <c r="G103" s="9" t="inlineStr">
+        <is>
+          <t>万吨</t>
+        </is>
+      </c>
+      <c r="H103" s="9" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I103" s="9" t="inlineStr">
+        <is>
+          <t>必须</t>
+        </is>
+      </c>
+      <c r="J103" s="9" t="inlineStr">
+        <is>
+          <t>派生汇总</t>
+        </is>
+      </c>
+      <c r="K103" s="9" t="inlineStr">
+        <is>
+          <t>计算</t>
+        </is>
+      </c>
+      <c r="L103" s="14" t="n"/>
+      <c r="M103" s="14" t="n"/>
+      <c r="N103" s="9" t="inlineStr">
+        <is>
+          <t>S5713307+S5713331+P5075301+U9895886+D2626009</t>
+        </is>
+      </c>
+      <c r="O103" s="9" t="inlineStr">
+        <is>
+          <t>螺纹+线材+热卷+冷轧+中厚板主要钢厂周产量求和</t>
+        </is>
+      </c>
+      <c r="P103" s="9" t="inlineStr">
+        <is>
+          <t>2020-02-07</t>
+        </is>
+      </c>
+      <c r="Q103" s="9" t="inlineStr">
+        <is>
+          <t>周五计算；周频有效</t>
+        </is>
+      </c>
+      <c r="R103" s="9" t="inlineStr">
+        <is>
+          <t>五大品种主要钢厂周度总产出</t>
+        </is>
+      </c>
     </row>
     <row r="104">
-      <c r="L104" s="15" t="n"/>
-      <c r="M104" s="15" t="n"/>
+      <c r="A104" s="9" t="inlineStr">
+        <is>
+          <t>TOTAL02</t>
+        </is>
+      </c>
+      <c r="B104" s="9" t="inlineStr">
+        <is>
+          <t>总供应</t>
+        </is>
+      </c>
+      <c r="C104" s="9" t="inlineStr">
+        <is>
+          <t>五大钢材社会库存合计</t>
+        </is>
+      </c>
+      <c r="D104" s="9" t="inlineStr">
+        <is>
+          <t>主要成材总社会库存</t>
+        </is>
+      </c>
+      <c r="E104" s="9" t="inlineStr">
+        <is>
+          <t>周</t>
+        </is>
+      </c>
+      <c r="F104" s="9" t="inlineStr">
+        <is>
+          <t>自有计算</t>
+        </is>
+      </c>
+      <c r="G104" s="9" t="inlineStr">
+        <is>
+          <t>万吨</t>
+        </is>
+      </c>
+      <c r="H104" s="9" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I104" s="9" t="inlineStr">
+        <is>
+          <t>必须</t>
+        </is>
+      </c>
+      <c r="J104" s="9" t="inlineStr">
+        <is>
+          <t>派生汇总</t>
+        </is>
+      </c>
+      <c r="K104" s="9" t="inlineStr">
+        <is>
+          <t>计算</t>
+        </is>
+      </c>
+      <c r="L104" s="14" t="n"/>
+      <c r="M104" s="14" t="n"/>
+      <c r="N104" s="9" t="inlineStr">
+        <is>
+          <t>H6924748+N5497850+X1924001+W2000685+W6382677</t>
+        </is>
+      </c>
+      <c r="O104" s="9" t="inlineStr">
+        <is>
+          <t>五大品种周度社会流通库存求和</t>
+        </is>
+      </c>
+      <c r="P104" s="9" t="inlineStr">
+        <is>
+          <t>2020-01-20</t>
+        </is>
+      </c>
+      <c r="Q104" s="9" t="inlineStr">
+        <is>
+          <t>周四计算；周频有效</t>
+        </is>
+      </c>
+      <c r="R104" s="9" t="inlineStr">
+        <is>
+          <t>五大主要钢材社会库存总量</t>
+        </is>
+      </c>
     </row>
     <row r="105">
-      <c r="L105" s="15" t="n"/>
-      <c r="M105" s="15" t="n"/>
+      <c r="A105" s="9" t="inlineStr">
+        <is>
+          <t>TOTAL03</t>
+        </is>
+      </c>
+      <c r="B105" s="9" t="inlineStr">
+        <is>
+          <t>总供应</t>
+        </is>
+      </c>
+      <c r="C105" s="9" t="inlineStr">
+        <is>
+          <t>五大钢材主要钢厂库存合计</t>
+        </is>
+      </c>
+      <c r="D105" s="9" t="inlineStr">
+        <is>
+          <t>主要成材总厂库</t>
+        </is>
+      </c>
+      <c r="E105" s="9" t="inlineStr">
+        <is>
+          <t>周</t>
+        </is>
+      </c>
+      <c r="F105" s="9" t="inlineStr">
+        <is>
+          <t>自有计算</t>
+        </is>
+      </c>
+      <c r="G105" s="9" t="inlineStr">
+        <is>
+          <t>万吨</t>
+        </is>
+      </c>
+      <c r="H105" s="9" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I105" s="9" t="inlineStr">
+        <is>
+          <t>必须</t>
+        </is>
+      </c>
+      <c r="J105" s="9" t="inlineStr">
+        <is>
+          <t>派生汇总</t>
+        </is>
+      </c>
+      <c r="K105" s="9" t="inlineStr">
+        <is>
+          <t>计算</t>
+        </is>
+      </c>
+      <c r="L105" s="14" t="n"/>
+      <c r="M105" s="14" t="n"/>
+      <c r="N105" s="9" t="inlineStr">
+        <is>
+          <t>R8579706+N2859772+L2776415+V9343799+C1585720</t>
+        </is>
+      </c>
+      <c r="O105" s="9" t="inlineStr">
+        <is>
+          <t>五大品种主要钢厂周度库存求和</t>
+        </is>
+      </c>
+      <c r="P105" s="9" t="inlineStr">
+        <is>
+          <t>2020-02-07</t>
+        </is>
+      </c>
+      <c r="Q105" s="9" t="inlineStr">
+        <is>
+          <t>周五计算；周频有效</t>
+        </is>
+      </c>
+      <c r="R105" s="9" t="inlineStr">
+        <is>
+          <t>主要钢厂成材厂库总规模</t>
+        </is>
+      </c>
     </row>
     <row r="106">
-      <c r="L106" s="15" t="n"/>
-      <c r="M106" s="15" t="n"/>
+      <c r="A106" s="9" t="inlineStr">
+        <is>
+          <t>TOTAL04</t>
+        </is>
+      </c>
+      <c r="B106" s="9" t="inlineStr">
+        <is>
+          <t>总供应</t>
+        </is>
+      </c>
+      <c r="C106" s="9" t="inlineStr">
+        <is>
+          <t>5大品种钢材社会库存(21城)</t>
+        </is>
+      </c>
+      <c r="D106" s="9" t="inlineStr">
+        <is>
+          <t>官方五大材社库总量</t>
+        </is>
+      </c>
+      <c r="E106" s="9" t="inlineStr">
+        <is>
+          <t>日</t>
+        </is>
+      </c>
+      <c r="F106" s="9" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G106" s="9" t="inlineStr">
+        <is>
+          <t>万吨</t>
+        </is>
+      </c>
+      <c r="H106" s="9" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I106" s="9" t="inlineStr">
+        <is>
+          <t>候选</t>
+        </is>
+      </c>
+      <c r="J106" s="9" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K106" s="9" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
+      <c r="L106" s="14" t="n"/>
+      <c r="M106" s="14" t="n"/>
+      <c r="N106" s="9" t="inlineStr">
+        <is>
+          <t>P7060164</t>
+        </is>
+      </c>
+      <c r="O106" s="9" t="inlineStr">
+        <is>
+          <t>中国:社会库存量:5大品种钢材(21个城市)</t>
+        </is>
+      </c>
+      <c r="P106" s="9" t="inlineStr">
+        <is>
+          <t>2020-01-10</t>
+        </is>
+      </c>
+      <c r="Q106" s="9" t="inlineStr">
+        <is>
+          <t>旬度发布 (标签为日频)</t>
+        </is>
+      </c>
+      <c r="R106" s="9" t="inlineStr">
+        <is>
+          <t>中钢协官方21个城市5大品种社会库存总量</t>
+        </is>
+      </c>
     </row>
     <row r="107">
-      <c r="L107" s="15" t="n"/>
-      <c r="M107" s="15" t="n"/>
+      <c r="A107" s="9" t="inlineStr">
+        <is>
+          <t>TOTAL05</t>
+        </is>
+      </c>
+      <c r="B107" s="9" t="inlineStr">
+        <is>
+          <t>总供应</t>
+        </is>
+      </c>
+      <c r="C107" s="9" t="inlineStr">
+        <is>
+          <t>重点钢铁企业钢材产量</t>
+        </is>
+      </c>
+      <c r="D107" s="9" t="inlineStr">
+        <is>
+          <t>官方重点钢企周度产出</t>
+        </is>
+      </c>
+      <c r="E107" s="9" t="inlineStr">
+        <is>
+          <t>周</t>
+        </is>
+      </c>
+      <c r="F107" s="9" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G107" s="9" t="inlineStr">
+        <is>
+          <t>万吨</t>
+        </is>
+      </c>
+      <c r="H107" s="9" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I107" s="9" t="inlineStr">
+        <is>
+          <t>候选</t>
+        </is>
+      </c>
+      <c r="J107" s="9" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K107" s="9" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
+      <c r="L107" s="14" t="n"/>
+      <c r="M107" s="14" t="n"/>
+      <c r="N107" s="9" t="inlineStr">
+        <is>
+          <t>D0194146</t>
+        </is>
+      </c>
+      <c r="O107" s="9" t="inlineStr">
+        <is>
+          <t>中国:产量:钢材:重点钢铁企业</t>
+        </is>
+      </c>
+      <c r="P107" s="9" t="inlineStr">
+        <is>
+          <t>2005-01-10</t>
+        </is>
+      </c>
+      <c r="Q107" s="9" t="inlineStr">
+        <is>
+          <t>旬/周度发布</t>
+        </is>
+      </c>
+      <c r="R107" s="9" t="inlineStr">
+        <is>
+          <t>中钢协重点钢铁企业钢材总产量</t>
+        </is>
+      </c>
     </row>
     <row r="108">
-      <c r="L108" s="15" t="n"/>
-      <c r="M108" s="15" t="n"/>
+      <c r="A108" s="9" t="inlineStr">
+        <is>
+          <t>ST01</t>
+        </is>
+      </c>
+      <c r="B108" s="9" t="inlineStr">
+        <is>
+          <t>现货</t>
+        </is>
+      </c>
+      <c r="C108" s="9" t="inlineStr">
+        <is>
+          <t>唐山热轧带钢现货价格</t>
+        </is>
+      </c>
+      <c r="D108" s="9" t="inlineStr">
+        <is>
+          <t>带钢现货基准</t>
+        </is>
+      </c>
+      <c r="E108" s="9" t="inlineStr">
+        <is>
+          <t>日</t>
+        </is>
+      </c>
+      <c r="F108" s="9" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G108" s="9" t="inlineStr">
+        <is>
+          <t>元/吨</t>
+        </is>
+      </c>
+      <c r="H108" s="9" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I108" s="9" t="inlineStr">
+        <is>
+          <t>候选</t>
+        </is>
+      </c>
+      <c r="J108" s="9" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K108" s="9" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
+      <c r="L108" s="14" t="n"/>
+      <c r="M108" s="14" t="n"/>
+      <c r="N108" s="9" t="inlineStr">
+        <is>
+          <t>S5705485</t>
+        </is>
+      </c>
+      <c r="O108" s="9" t="inlineStr">
+        <is>
+          <t>中国:唐山:价格:热轧带钢(2.5mm*232)</t>
+        </is>
+      </c>
+      <c r="P108" s="9" t="inlineStr">
+        <is>
+          <t>2009-08-03</t>
+        </is>
+      </c>
+      <c r="Q108" s="9" t="inlineStr">
+        <is>
+          <t>每个交易日更新；日频有效</t>
+        </is>
+      </c>
+      <c r="R108" s="9" t="inlineStr">
+        <is>
+          <t>唐山窄带主流现货基准日价</t>
+        </is>
+      </c>
     </row>
     <row r="109">
-      <c r="L109" s="15" t="n"/>
-      <c r="M109" s="15" t="n"/>
+      <c r="A109" s="9" t="inlineStr">
+        <is>
+          <t>GI01</t>
+        </is>
+      </c>
+      <c r="B109" s="9" t="inlineStr">
+        <is>
+          <t>热卷</t>
+        </is>
+      </c>
+      <c r="C109" s="9" t="inlineStr">
+        <is>
+          <t>重点企业镀锌板累计产量</t>
+        </is>
+      </c>
+      <c r="D109" s="9" t="inlineStr">
+        <is>
+          <t>冷轧下游深加工产出</t>
+        </is>
+      </c>
+      <c r="E109" s="9" t="inlineStr">
+        <is>
+          <t>月</t>
+        </is>
+      </c>
+      <c r="F109" s="9" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G109" s="9" t="inlineStr">
+        <is>
+          <t>万吨</t>
+        </is>
+      </c>
+      <c r="H109" s="9" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I109" s="9" t="inlineStr">
+        <is>
+          <t>候选</t>
+        </is>
+      </c>
+      <c r="J109" s="9" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K109" s="9" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
+      <c r="L109" s="14" t="n"/>
+      <c r="M109" s="14" t="n"/>
+      <c r="N109" s="9" t="inlineStr">
+        <is>
+          <t>S0114079</t>
+        </is>
+      </c>
+      <c r="O109" s="9" t="inlineStr">
+        <is>
+          <t>中国:产量:镀锌板(带):重点企业:累计值</t>
+        </is>
+      </c>
+      <c r="P109" s="9" t="inlineStr">
+        <is>
+          <t>2005-01-31</t>
+        </is>
+      </c>
+      <c r="Q109" s="9" t="inlineStr">
+        <is>
+          <t>月度发布；月频有效</t>
+        </is>
+      </c>
+      <c r="R109" s="9" t="inlineStr">
+        <is>
+          <t>中钢协重点钢铁企业镀锌板带累计产量</t>
+        </is>
+      </c>
     </row>
     <row r="110">
-      <c r="L110" s="15" t="n"/>
-      <c r="M110" s="15" t="n"/>
+      <c r="A110" s="9" t="inlineStr">
+        <is>
+          <t>GI02</t>
+        </is>
+      </c>
+      <c r="B110" s="9" t="inlineStr">
+        <is>
+          <t>热卷</t>
+        </is>
+      </c>
+      <c r="C110" s="9" t="inlineStr">
+        <is>
+          <t>全国镀锌板库存量</t>
+        </is>
+      </c>
+      <c r="D110" s="9" t="inlineStr">
+        <is>
+          <t>深加工成材库存</t>
+        </is>
+      </c>
+      <c r="E110" s="9" t="inlineStr">
+        <is>
+          <t>月</t>
+        </is>
+      </c>
+      <c r="F110" s="9" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G110" s="9" t="inlineStr">
+        <is>
+          <t>万吨</t>
+        </is>
+      </c>
+      <c r="H110" s="9" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I110" s="9" t="inlineStr">
+        <is>
+          <t>候选</t>
+        </is>
+      </c>
+      <c r="J110" s="9" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K110" s="9" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
+      <c r="L110" s="14" t="n"/>
+      <c r="M110" s="14" t="n"/>
+      <c r="N110" s="9" t="inlineStr">
+        <is>
+          <t>S0066739</t>
+        </is>
+      </c>
+      <c r="O110" s="9" t="inlineStr">
+        <is>
+          <t>中国:库存量:镀锌板(带)</t>
+        </is>
+      </c>
+      <c r="P110" s="9" t="inlineStr">
+        <is>
+          <t>2005-01-31</t>
+        </is>
+      </c>
+      <c r="Q110" s="9" t="inlineStr">
+        <is>
+          <t>月度发布；月频有效</t>
+        </is>
+      </c>
+      <c r="R110" s="9" t="inlineStr">
+        <is>
+          <t>全国镀锌板月度总库存</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="L111" s="15" t="n"/>

</xml_diff>

<commit_message>
feat(data): add 28 raw materials and thermal coal indicators to A03 data map
</commit_message>
<xml_diff>
--- a/outputs/阶段A_框架初版/A03_数据地图.xlsx
+++ b/outputs/阶段A_框架初版/A03_数据地图.xlsx
@@ -185,7 +185,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Register1" displayName="Register1" ref="A5:R110" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Register1" displayName="Register1" ref="A5:R138" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <tableColumns count="18">
     <tableColumn id="1" name="变量ID"/>
     <tableColumn id="2" name="模块"/>
@@ -9357,116 +9357,2356 @@
       </c>
     </row>
     <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>FR01</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>原料</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>CDFI西澳丹皮尔-青岛海运费</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>BCI C5西澳铁矿石航线核心运费，长流程原料到港成本关键构成</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>日</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>美元/吨</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>必须</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
       <c r="L111" s="15" t="n"/>
       <c r="M111" s="15" t="n"/>
+      <c r="N111" t="inlineStr">
+        <is>
+          <t>S0176220</t>
+        </is>
+      </c>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>中国进口干散货运价指数:海岬型船:铁矿石:西澳大利亚丹皮尔-青岛</t>
+        </is>
+      </c>
+      <c r="P111" t="inlineStr">
+        <is>
+          <t>2012-11-28</t>
+        </is>
+      </c>
+      <c r="Q111" t="inlineStr">
+        <is>
+          <t>交易日更新；日频有效</t>
+        </is>
+      </c>
+      <c r="R111" t="inlineStr">
+        <is>
+          <t>上海航运交易所CDFI官方序列；长流程铁矿进口运费核心定价标的</t>
+        </is>
+      </c>
     </row>
     <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>FR02</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>原料</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>CDFI巴西图巴朗-青岛海运费</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>BCI C3巴西铁矿石长航线运费，波动弹性大，衡量全球运力紧缩程度</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>日</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>美元/吨</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>必须</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
       <c r="L112" s="15" t="n"/>
       <c r="M112" s="15" t="n"/>
+      <c r="N112" t="inlineStr">
+        <is>
+          <t>S0176221</t>
+        </is>
+      </c>
+      <c r="O112" t="inlineStr">
+        <is>
+          <t>中国进口干散货运价指数:海岬型船:铁矿石:巴西图巴朗-青岛</t>
+        </is>
+      </c>
+      <c r="P112" t="inlineStr">
+        <is>
+          <t>2012-11-28</t>
+        </is>
+      </c>
+      <c r="Q112" t="inlineStr">
+        <is>
+          <t>交易日更新；日频有效</t>
+        </is>
+      </c>
+      <c r="R112" t="inlineStr">
+        <is>
+          <t>上海航运交易所CDFI官方序列；巴西淡水河谷长航线运费弹性指标</t>
+        </is>
+      </c>
     </row>
     <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>FR03</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>原料</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>CDFI海岬型船铁矿石运价指数</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>中国进口铁矿石海岬型船综合运价指数</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>日</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>点</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>候选</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
       <c r="L113" s="15" t="n"/>
       <c r="M113" s="15" t="n"/>
+      <c r="N113" t="inlineStr">
+        <is>
+          <t>S0266069</t>
+        </is>
+      </c>
+      <c r="O113" t="inlineStr">
+        <is>
+          <t>中国进口干散货运价指数:海岬型船:铁矿石</t>
+        </is>
+      </c>
+      <c r="P113" t="inlineStr">
+        <is>
+          <t>2017-11-28</t>
+        </is>
+      </c>
+      <c r="Q113" t="inlineStr">
+        <is>
+          <t>交易日更新；日频有效</t>
+        </is>
+      </c>
+      <c r="R113" t="inlineStr">
+        <is>
+          <t>综合反映中国港口海岬型铁矿船平均运价走势</t>
+        </is>
+      </c>
     </row>
     <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>FR04</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>原料</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>中国进口干散货运价综合指数</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>CDFI综合指数，反映铁矿、煤炭、大豆等大宗干散货进口总体运输成本</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>日</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>点</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>候选</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
       <c r="L114" s="15" t="n"/>
       <c r="M114" s="15" t="n"/>
+      <c r="N114" t="inlineStr">
+        <is>
+          <t>S0205030</t>
+        </is>
+      </c>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>中国进口干散货运价指数:综合指数</t>
+        </is>
+      </c>
+      <c r="P114" t="inlineStr">
+        <is>
+          <t>2013-11-28</t>
+        </is>
+      </c>
+      <c r="Q114" t="inlineStr">
+        <is>
+          <t>交易日更新；日频有效</t>
+        </is>
+      </c>
+      <c r="R114" t="inlineStr">
+        <is>
+          <t>上海航运交易所编制的干散货综合运费指数</t>
+        </is>
+      </c>
     </row>
     <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>FR05</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>宏观</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>波罗的海干散货指数(BDI)</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>全球大宗商品航运景气度与国际宏观贸易总需求晴雨表</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>日</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>点</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>必须</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
       <c r="L115" s="15" t="n"/>
       <c r="M115" s="15" t="n"/>
+      <c r="N115" t="inlineStr">
+        <is>
+          <t>S0031550</t>
+        </is>
+      </c>
+      <c r="O115" t="inlineStr">
+        <is>
+          <t>波罗的海干散货指数(BDI)</t>
+        </is>
+      </c>
+      <c r="P115" t="inlineStr">
+        <is>
+          <t>1988-10-19</t>
+        </is>
+      </c>
+      <c r="Q115" t="inlineStr">
+        <is>
+          <t>交易日更新；日频有效</t>
+        </is>
+      </c>
+      <c r="R115" t="inlineStr">
+        <is>
+          <t>波罗的海交易所基准；全球宏观工业需求及大宗物流先行指标</t>
+        </is>
+      </c>
     </row>
     <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>IO01</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>现货</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>青岛港PB粉车板价(含税)</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>铁矿石现货基差与盘面交易的核心定价锚（61.5%澳粉主流标的）</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>日</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>元/湿吨</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>必须</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
       <c r="L116" s="15" t="n"/>
       <c r="M116" s="15" t="n"/>
+      <c r="N116" t="inlineStr">
+        <is>
+          <t>S0174655</t>
+        </is>
+      </c>
+      <c r="O116" t="inlineStr">
+        <is>
+          <t>中国:青岛港:车板价:PB粉矿(61.5%,澳大利亚)</t>
+        </is>
+      </c>
+      <c r="P116" t="inlineStr">
+        <is>
+          <t>2011-09-08</t>
+        </is>
+      </c>
+      <c r="Q116" t="inlineStr">
+        <is>
+          <t>每个交易日更新；日频有效</t>
+        </is>
+      </c>
+      <c r="R116" t="inlineStr">
+        <is>
+          <t>国内港口现货成交量最大、期货盘面基差锚定标的</t>
+        </is>
+      </c>
     </row>
     <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>IO02</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>原料</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>唐山迁安铁精粉市场价</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>国产精粉核心基准（湿基不含税66%），长流程内矿配比调节信号</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>日</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>元/吨</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>待核实</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>候选</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
       <c r="L117" s="15" t="n"/>
       <c r="M117" s="15" t="n"/>
+      <c r="N117" t="inlineStr">
+        <is>
+          <t>A3695347</t>
+        </is>
+      </c>
+      <c r="O117" t="inlineStr">
+        <is>
+          <t>中国:迁安:市场价(湿基不含税):铁精粉(0.66)</t>
+        </is>
+      </c>
+      <c r="P117" t="inlineStr">
+        <is>
+          <t>2017-01-01</t>
+        </is>
+      </c>
+      <c r="Q117" t="inlineStr">
+        <is>
+          <t>工作日更新；日频有效</t>
+        </is>
+      </c>
+      <c r="R117" t="inlineStr">
+        <is>
+          <t>百川盈孚专区；国内高品位内矿价格风向标</t>
+        </is>
+      </c>
     </row>
     <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>IO03</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>原料</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>铁矿石价格指数(62%,FOB)</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>国际美金离岸价指数，测算内外矿进口倒挂/顺差利润</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>日</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>美元/吨</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>待核实</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>候选</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
       <c r="L118" s="15" t="n"/>
       <c r="M118" s="15" t="n"/>
+      <c r="N118" t="inlineStr">
+        <is>
+          <t>S5716219</t>
+        </is>
+      </c>
+      <c r="O118" t="inlineStr">
+        <is>
+          <t>中国:铁矿石价格指数(62%,FOB)</t>
+        </is>
+      </c>
+      <c r="P118" t="inlineStr">
+        <is>
+          <t>2019-09-27</t>
+        </is>
+      </c>
+      <c r="Q118" t="inlineStr">
+        <is>
+          <t>工作日更新；日频有效</t>
+        </is>
+      </c>
+      <c r="R118" t="inlineStr">
+        <is>
+          <t>唐宋钢铁在线；海外铁矿离岸美金计价</t>
+        </is>
+      </c>
     </row>
     <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>JM01</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>原料</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>甘其毛都蒙5#焦煤出厂价</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>蒙古通关核心品种（A≤10%,S0.6%,G≥80），边际焦煤供给最灵敏定价</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>日</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>元/吨</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>待核实</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>必须</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
       <c r="L119" s="15" t="n"/>
       <c r="M119" s="15" t="n"/>
+      <c r="N119" t="inlineStr">
+        <is>
+          <t>U1034836</t>
+        </is>
+      </c>
+      <c r="O119" t="inlineStr">
+        <is>
+          <t>蒙古:出厂价:焦煤(5#,A≤10%,V26-28%,S0.6%,G≥80,Mt≤10%,CSR60%,甘其毛都口岸)</t>
+        </is>
+      </c>
+      <c r="P119" t="inlineStr">
+        <is>
+          <t>2024-05-20</t>
+        </is>
+      </c>
+      <c r="Q119" t="inlineStr">
+        <is>
+          <t>工作日更新；日频有效</t>
+        </is>
+      </c>
+      <c r="R119" t="inlineStr">
+        <is>
+          <t>钢之家专区；中蒙陆路口岸最核心通关提货现货价</t>
+        </is>
+      </c>
     </row>
     <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>JM02</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>原料</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>唐山沙河驿蒙焦煤到厂价</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>蒙煤运抵河北钢焦集群提货价，反映蒙煤内陆分销与运输成本</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>日</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>元/吨</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>待核实</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>候选</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
       <c r="L120" s="15" t="n"/>
       <c r="M120" s="15" t="n"/>
+      <c r="N120" t="inlineStr">
+        <is>
+          <t>B4120932</t>
+        </is>
+      </c>
+      <c r="O120" t="inlineStr">
+        <is>
+          <t>蒙古:出厂价:焦煤(A≤10.5%,V26-28%,S0.6%,G≥80,Mt≤10%,CSR60%,唐山沙河驿产)</t>
+        </is>
+      </c>
+      <c r="P120" t="inlineStr">
+        <is>
+          <t>2016-11-25</t>
+        </is>
+      </c>
+      <c r="Q120" t="inlineStr">
+        <is>
+          <t>工作日更新；日频有效</t>
+        </is>
+      </c>
+      <c r="R120" t="inlineStr">
+        <is>
+          <t>钢之家专区；历史序列长(自2016年)，唐山主要蒙煤交割分销基准</t>
+        </is>
+      </c>
     </row>
     <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>JM03</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>原料</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>山西主焦煤平均价</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>山西核心产地优质低硫/高硫主焦煤综合价格，内煤定价中枢</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>日</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>元/吨</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>待核实</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>必须</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
       <c r="L121" s="15" t="n"/>
       <c r="M121" s="15" t="n"/>
+      <c r="N121" t="inlineStr">
+        <is>
+          <t>S5132022</t>
+        </is>
+      </c>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>中国:山西:平均价:主焦煤</t>
+        </is>
+      </c>
+      <c r="P121" t="inlineStr">
+        <is>
+          <t>2016-01-04</t>
+        </is>
+      </c>
+      <c r="Q121" t="inlineStr">
+        <is>
+          <t>工作日更新；日频有效</t>
+        </is>
+      </c>
+      <c r="R121" t="inlineStr">
+        <is>
+          <t>钢之家专区；山西省内主流矿区主焦煤现货均价</t>
+        </is>
+      </c>
     </row>
     <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>JM04</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>原料</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>澳大利亚峰景矿焦煤到岸价</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>国际最高品质硬焦煤基准（CSR74%），衡量海内外焦煤价差与进口窗口</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>日</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>美元/吨</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>待核实</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>候选</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
       <c r="L122" s="15" t="n"/>
       <c r="M122" s="15" t="n"/>
+      <c r="N122" t="inlineStr">
+        <is>
+          <t>S5120155</t>
+        </is>
+      </c>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t>中国:现货价(到岸价):焦煤(峰景矿,A:10.5%,V:21.5%,S:0.61%,G:87,Y:19,Mt:10%,CSR74%,澳大利亚产)</t>
+        </is>
+      </c>
+      <c r="P122" t="inlineStr">
+        <is>
+          <t>2012-11-11</t>
+        </is>
+      </c>
+      <c r="Q122" t="inlineStr">
+        <is>
+          <t>工作日更新；日频有效</t>
+        </is>
+      </c>
+      <c r="R122" t="inlineStr">
+        <is>
+          <t>钢之家专区；海运顶级低挥发炼焦煤CIF基准</t>
+        </is>
+      </c>
     </row>
     <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>JM05</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>原料</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>焦煤现货领先价格指数</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Wind编制的焦煤现货领先价格指数，提供敏捷价格信号</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>日</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>元/吨</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>候选</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
       <c r="L123" s="15" t="n"/>
       <c r="M123" s="15" t="n"/>
+      <c r="N123" t="inlineStr">
+        <is>
+          <t>U4421912</t>
+        </is>
+      </c>
+      <c r="O123" t="inlineStr">
+        <is>
+          <t>中国:现货领先价格:焦煤</t>
+        </is>
+      </c>
+      <c r="P123" t="inlineStr">
+        <is>
+          <t>2019-01-01</t>
+        </is>
+      </c>
+      <c r="Q123" t="inlineStr">
+        <is>
+          <t>交易日更新；日频有效</t>
+        </is>
+      </c>
+      <c r="R123" t="inlineStr">
+        <is>
+          <t>Wind自编指数；先导性价格跟踪</t>
+        </is>
+      </c>
     </row>
     <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>J01</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>现货</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>日照港准一级冶金焦平仓价</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>期货最核心交割对标标的（A13,S0.7,CSR60,含税），贸易蓄水池风向标</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>日</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>元/吨</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>必须</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
       <c r="L124" s="15" t="n"/>
       <c r="M124" s="15" t="n"/>
+      <c r="N124" t="inlineStr">
+        <is>
+          <t>S5134898</t>
+        </is>
+      </c>
+      <c r="O124" t="inlineStr">
+        <is>
+          <t>中国:日照港:平仓价(含税):冶金焦(准一级,A13,S0.7,CSR60,MT7)</t>
+        </is>
+      </c>
+      <c r="P124" t="inlineStr">
+        <is>
+          <t>2017-06-13</t>
+        </is>
+      </c>
+      <c r="Q124" t="inlineStr">
+        <is>
+          <t>每个交易日更新；日频有效</t>
+        </is>
+      </c>
+      <c r="R124" t="inlineStr">
+        <is>
+          <t>Wind自采；大商所焦炭期货最核心交割基准对齐港口价</t>
+        </is>
+      </c>
     </row>
     <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>J02</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>原料</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>日照港准一级冶金焦市场价</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>港口贸易商现货主流报价，与平仓价交叉印证流动性折溢价</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>日</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>元/吨</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>待核实</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>候选</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
       <c r="L125" s="15" t="n"/>
       <c r="M125" s="15" t="n"/>
+      <c r="N125" t="inlineStr">
+        <is>
+          <t>P8829103</t>
+        </is>
+      </c>
+      <c r="O125" t="inlineStr">
+        <is>
+          <t>中国:日照港:市场价:冶金焦(准一级,A&lt;13.0%,S&lt;0.7%,Mt:0%,M25&gt;90%,CSR&gt;60%,华北,贸易商)</t>
+        </is>
+      </c>
+      <c r="P125" t="inlineStr">
+        <is>
+          <t>2024-05-20</t>
+        </is>
+      </c>
+      <c r="Q125" t="inlineStr">
+        <is>
+          <t>工作日更新；日频有效</t>
+        </is>
+      </c>
+      <c r="R125" t="inlineStr">
+        <is>
+          <t>钢之家专区；日照港贸易商主流成交与报价</t>
+        </is>
+      </c>
     </row>
     <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>J03</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>成本利润</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>全国焦炭生产毛利</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>独立焦化厂吨焦盈利状态，判断焦炭提涨/提降博弈和限产意愿</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>周</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>元/吨</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>待核实</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>必须</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
       <c r="L126" s="15" t="n"/>
       <c r="M126" s="15" t="n"/>
+      <c r="N126" t="inlineStr">
+        <is>
+          <t>S9985549</t>
+        </is>
+      </c>
+      <c r="O126" t="inlineStr">
+        <is>
+          <t>中国:毛利:焦炭</t>
+        </is>
+      </c>
+      <c r="P126" t="inlineStr">
+        <is>
+          <t>2017-01-06</t>
+        </is>
+      </c>
+      <c r="Q126" t="inlineStr">
+        <is>
+          <t>周五更新；周频有效</t>
+        </is>
+      </c>
+      <c r="R126" t="inlineStr">
+        <is>
+          <t>百川盈孚专区；判断焦炭提涨/提降产业博弈节奏的核心指标</t>
+        </is>
+      </c>
     </row>
     <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>TC01</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>原料</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>秦皇岛港动力煤平仓价(Q5500)</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>全国动力煤现货定价总锚（5500大卡长协与现货基准）</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>周</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>元/吨</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>必须</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
       <c r="L127" s="15" t="n"/>
       <c r="M127" s="15" t="n"/>
+      <c r="N127" t="inlineStr">
+        <is>
+          <t>S5104572</t>
+        </is>
+      </c>
+      <c r="O127" t="inlineStr">
+        <is>
+          <t>中国:秦皇岛港:平仓价:动力煤(Q5500K)</t>
+        </is>
+      </c>
+      <c r="P127" t="inlineStr">
+        <is>
+          <t>2003-02-28</t>
+        </is>
+      </c>
+      <c r="Q127" t="inlineStr">
+        <is>
+          <t>周三更新；周频有效</t>
+        </is>
+      </c>
+      <c r="R127" t="inlineStr">
+        <is>
+          <t>秦皇岛煤炭网；煤炭行业最核心定价总中枢</t>
+        </is>
+      </c>
     </row>
     <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>TC02</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>原料</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>秦皇岛动力煤市场价(Q5500)</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>日频动力煤现货报价，提供敏捷日度波动跟踪</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>日</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>元/吨</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>待核实</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>候选</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
       <c r="L128" s="15" t="n"/>
       <c r="M128" s="15" t="n"/>
+      <c r="N128" t="inlineStr">
+        <is>
+          <t>S9983507</t>
+        </is>
+      </c>
+      <c r="O128" t="inlineStr">
+        <is>
+          <t>中国:秦皇岛:市场价(含税):动力煤(Q5500)</t>
+        </is>
+      </c>
+      <c r="P128" t="inlineStr">
+        <is>
+          <t>2017-01-01</t>
+        </is>
+      </c>
+      <c r="Q128" t="inlineStr">
+        <is>
+          <t>工作日更新；日频有效</t>
+        </is>
+      </c>
+      <c r="R128" t="inlineStr">
+        <is>
+          <t>百川盈孚专区；日频动力煤港口现货跟踪</t>
+        </is>
+      </c>
     </row>
     <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>TC03</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>原料</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>鄂尔多斯动力煤车板价(Q5500)</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>动力煤最大产区坑口/车板基准，监控产地-港口发运发运倒挂</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>周</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>元/吨</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>必须</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
       <c r="L129" s="15" t="n"/>
       <c r="M129" s="15" t="n"/>
+      <c r="N129" t="inlineStr">
+        <is>
+          <t>S5133608</t>
+        </is>
+      </c>
+      <c r="O129" t="inlineStr">
+        <is>
+          <t>中国:鄂尔多斯:车板价:动力煤(Q5500)</t>
+        </is>
+      </c>
+      <c r="P129" t="inlineStr">
+        <is>
+          <t>2014-09-30</t>
+        </is>
+      </c>
+      <c r="Q129" t="inlineStr">
+        <is>
+          <t>周一更新；周频有效</t>
+        </is>
+      </c>
+      <c r="R129" t="inlineStr">
+        <is>
+          <t>中国煤炭市场网；内蒙古主产区坑口与车板定价</t>
+        </is>
+      </c>
     </row>
     <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>TC04</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>原料</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>秦皇岛港煤炭库存量</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>北方第一大煤炭下水港蓄水池，港口疏港与集港拥堵指标</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>日</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>万吨</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>必须</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
       <c r="L130" s="15" t="n"/>
       <c r="M130" s="15" t="n"/>
+      <c r="N130" t="inlineStr">
+        <is>
+          <t>S5103725</t>
+        </is>
+      </c>
+      <c r="O130" t="inlineStr">
+        <is>
+          <t>中国:秦皇岛港:库存量:煤炭</t>
+        </is>
+      </c>
+      <c r="P130" t="inlineStr">
+        <is>
+          <t>2002-01-23</t>
+        </is>
+      </c>
+      <c r="Q130" t="inlineStr">
+        <is>
+          <t>每日更新；日频有效</t>
+        </is>
+      </c>
+      <c r="R130" t="inlineStr">
+        <is>
+          <t>秦皇岛煤炭网；最敏捷的动力煤中转枢纽蓄水池指标</t>
+        </is>
+      </c>
     </row>
     <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>TC05</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>原料</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>重点电厂煤炭库存量</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>下游终端火电企业总库存量，判断电厂补库与去库周期</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>周</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>万吨</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>必须</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
       <c r="L131" s="15" t="n"/>
       <c r="M131" s="15" t="n"/>
+      <c r="N131" t="inlineStr">
+        <is>
+          <t>V2000618</t>
+        </is>
+      </c>
+      <c r="O131" t="inlineStr">
+        <is>
+          <t>中国:库存量:煤炭重点电厂</t>
+        </is>
+      </c>
+      <c r="P131" t="inlineStr">
+        <is>
+          <t>2022-01-13</t>
+        </is>
+      </c>
+      <c r="Q131" t="inlineStr">
+        <is>
+          <t>周度更新；周频有效</t>
+        </is>
+      </c>
+      <c r="R131" t="inlineStr">
+        <is>
+          <t>根据新闻整理；全国主要统调/重点电厂存煤总量</t>
+        </is>
+      </c>
     </row>
     <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>TC06</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>原料</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>重点电厂煤炭日耗量</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>下游火电实际耗煤强度，迎峰度夏/度冬需求景气度真实度量</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>周</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>万吨</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>必须</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
       <c r="L132" s="15" t="n"/>
       <c r="M132" s="15" t="n"/>
+      <c r="N132" t="inlineStr">
+        <is>
+          <t>Q0149884</t>
+        </is>
+      </c>
+      <c r="O132" t="inlineStr">
+        <is>
+          <t>中国:日耗量:煤炭重点电厂</t>
+        </is>
+      </c>
+      <c r="P132" t="inlineStr">
+        <is>
+          <t>2022-01-13</t>
+        </is>
+      </c>
+      <c r="Q132" t="inlineStr">
+        <is>
+          <t>周度更新；周频有效</t>
+        </is>
+      </c>
+      <c r="R132" t="inlineStr">
+        <is>
+          <t>根据新闻整理；度量下游工业与居民用电耗煤强度</t>
+        </is>
+      </c>
     </row>
     <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>TC07</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>原料</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>重点电厂煤炭库存可用天数</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>库耗比核心指标，直接决定电厂采购紧迫度与煤价拐点</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>周</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>天</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>必须</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
       <c r="L133" s="15" t="n"/>
       <c r="M133" s="15" t="n"/>
+      <c r="N133" t="inlineStr">
+        <is>
+          <t>C2918730</t>
+        </is>
+      </c>
+      <c r="O133" t="inlineStr">
+        <is>
+          <t>中国:库存可用天数:煤炭重点电厂</t>
+        </is>
+      </c>
+      <c r="P133" t="inlineStr">
+        <is>
+          <t>2022-01-13</t>
+        </is>
+      </c>
+      <c r="Q133" t="inlineStr">
+        <is>
+          <t>周度更新；周频有效</t>
+        </is>
+      </c>
+      <c r="R133" t="inlineStr">
+        <is>
+          <t>根据新闻整理；电厂存煤天数低于安全线(15天)将触发紧急补库</t>
+        </is>
+      </c>
     </row>
     <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>TC08</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>原料</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>纽卡斯尔-舟山海岬型煤炭运费</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>澳大利亚进口海运煤运费，与铁矿航运形成跨品种运力竞争分析</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>日</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>美元/吨</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>候选</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
       <c r="L134" s="15" t="n"/>
       <c r="M134" s="15" t="n"/>
+      <c r="N134" t="inlineStr">
+        <is>
+          <t>S0176223</t>
+        </is>
+      </c>
+      <c r="O134" t="inlineStr">
+        <is>
+          <t>中国进口干散货运价指数:海岬型船:煤炭:澳大利亚纽卡斯尔-舟山</t>
+        </is>
+      </c>
+      <c r="P134" t="inlineStr">
+        <is>
+          <t>2012-11-28</t>
+        </is>
+      </c>
+      <c r="Q134" t="inlineStr">
+        <is>
+          <t>交易日更新；日频有效</t>
+        </is>
+      </c>
+      <c r="R134" t="inlineStr">
+        <is>
+          <t>上海航运交易所CDFI官方序列；主要海运进口煤航线</t>
+        </is>
+      </c>
     </row>
     <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>B07</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>现货</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>江苏普碳方坯价格</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>华东钢坯现货基准（20MnSi），监控南北坯料跨区套利价差</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>日</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>元/吨</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>必须</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
       <c r="L135" s="15" t="n"/>
       <c r="M135" s="15" t="n"/>
+      <c r="N135" t="inlineStr">
+        <is>
+          <t>S0143502</t>
+        </is>
+      </c>
+      <c r="O135" t="inlineStr">
+        <is>
+          <t>中国:江苏:价格:方坯(20MnSi)</t>
+        </is>
+      </c>
+      <c r="P135" t="inlineStr">
+        <is>
+          <t>2007-01-31</t>
+        </is>
+      </c>
+      <c r="Q135" t="inlineStr">
+        <is>
+          <t>每个交易日更新；日频有效</t>
+        </is>
+      </c>
+      <c r="R135" t="inlineStr">
+        <is>
+          <t>Wind自采；华东江浙沪调坯厂与长流程钢企坯料价格</t>
+        </is>
+      </c>
     </row>
     <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>SC01</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>现货</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>张家港废钢市场价(6-8mm)</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>华东重废现货风向标（不含税），紧跟沙钢周边回收与加工成本</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>日</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>元/吨</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>必须</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
       <c r="L136" s="15" t="n"/>
       <c r="M136" s="15" t="n"/>
+      <c r="N136" t="inlineStr">
+        <is>
+          <t>S5712502</t>
+        </is>
+      </c>
+      <c r="O136" t="inlineStr">
+        <is>
+          <t>中国:张家港:市场价(不含税):废钢(6-8mm)</t>
+        </is>
+      </c>
+      <c r="P136" t="inlineStr">
+        <is>
+          <t>2012-06-05</t>
+        </is>
+      </c>
+      <c r="Q136" t="inlineStr">
+        <is>
+          <t>每个交易日更新；日频有效</t>
+        </is>
+      </c>
+      <c r="R136" t="inlineStr">
+        <is>
+          <t>Wind自采；华东废钢主集散地现货重废价格</t>
+        </is>
+      </c>
     </row>
     <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>SC02</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>现货</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>唐山废钢市场价(6-8mm)</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>华北唐山长流程转炉加废现货价格，衡量高炉铁水与废钢比价</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>日</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>元/吨</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>可获得</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>必须</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
       <c r="L137" s="15" t="n"/>
       <c r="M137" s="15" t="n"/>
+      <c r="N137" t="inlineStr">
+        <is>
+          <t>S5700017</t>
+        </is>
+      </c>
+      <c r="O137" t="inlineStr">
+        <is>
+          <t>中国:唐山:市场价(不含税):废钢(6-8mm)</t>
+        </is>
+      </c>
+      <c r="P137" t="inlineStr">
+        <is>
+          <t>2007-01-04</t>
+        </is>
+      </c>
+      <c r="Q137" t="inlineStr">
+        <is>
+          <t>每个交易日更新；日频有效</t>
+        </is>
+      </c>
+      <c r="R137" t="inlineStr">
+        <is>
+          <t>Wind自采；华北高炉转炉废钢配比调节成本锚</t>
+        </is>
+      </c>
     </row>
     <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>SC03</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>现货</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>沙钢重废采购价格(三类≥6mm)</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>沙钢官方采购执行调价，全国短流程电炉厂废钢定价风向标</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>日</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>Wind EDB</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>元/吨</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>待核实</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>必须</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>直接观测</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>原始</t>
+        </is>
+      </c>
       <c r="L138" s="15" t="n"/>
       <c r="M138" s="15" t="n"/>
+      <c r="N138" t="inlineStr">
+        <is>
+          <t>S9973428</t>
+        </is>
+      </c>
+      <c r="O138" t="inlineStr">
+        <is>
+          <t>富宝:中国:价格(13%税):重废(三类,≥6mm):沙钢</t>
+        </is>
+      </c>
+      <c r="P138" t="inlineStr">
+        <is>
+          <t>2006-01-24</t>
+        </is>
+      </c>
+      <c r="Q138" t="inlineStr">
+        <is>
+          <t>每日更新；日频有效</t>
+        </is>
+      </c>
+      <c r="R138" t="inlineStr">
+        <is>
+          <t>富宝资讯专区；国内废钢最核心的钢厂挂牌采购定价基准</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="L139" s="15" t="n"/>

</xml_diff>